<commit_message>
change saving of auth codes
</commit_message>
<xml_diff>
--- a/static/img/logo.xlsx
+++ b/static/img/logo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Desktop\repos\korshiles\static\img\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F147EDD2-CBEF-4E44-83B1-348E76533748}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A67AA6-DE8D-470E-A828-28675CEECDF7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17670" yWindow="1695" windowWidth="10500" windowHeight="12375" xr2:uid="{D5EB7962-FF30-4317-BC7E-7FE01F0EE3A6}"/>
+    <workbookView xWindow="22590" yWindow="1440" windowWidth="6300" windowHeight="12375" xr2:uid="{D5EB7962-FF30-4317-BC7E-7FE01F0EE3A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -418,7 +418,7 @@
         <v>0</v>
       </c>
       <c r="B1">
-        <v>800</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -426,7 +426,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>800</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -435,7 +435,7 @@
       </c>
       <c r="B4">
         <f>B1/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -444,7 +444,7 @@
       </c>
       <c r="B5">
         <f>B2/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -453,7 +453,7 @@
       </c>
       <c r="B6">
         <f>B1/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -462,7 +462,7 @@
       </c>
       <c r="B8">
         <f>B1/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -471,7 +471,7 @@
       </c>
       <c r="B9">
         <f>B2/3.2</f>
-        <v>250</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -480,7 +480,7 @@
       </c>
       <c r="B10">
         <f>(B1-B8)/2</f>
-        <v>200</v>
+        <v>256</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -489,7 +489,7 @@
       </c>
       <c r="B11">
         <f>B2/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -498,7 +498,7 @@
       </c>
       <c r="B14">
         <f>B1/20</f>
-        <v>40</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -507,11 +507,11 @@
       </c>
       <c r="B15">
         <f>B1/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
       <c r="C15">
         <f>B2/5</f>
-        <v>160</v>
+        <v>204.8</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -520,11 +520,11 @@
       </c>
       <c r="B16">
         <f>B10-B14</f>
-        <v>160</v>
+        <v>204.8</v>
       </c>
       <c r="C16">
         <f>B2/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -533,11 +533,11 @@
       </c>
       <c r="B17">
         <f>B10+B8+B14</f>
-        <v>640</v>
+        <v>819.2</v>
       </c>
       <c r="C17">
         <f>B2/2</f>
-        <v>400</v>
+        <v>512</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -546,7 +546,7 @@
       </c>
       <c r="B20">
         <f>B1/80</f>
-        <v>10</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -555,7 +555,7 @@
       </c>
       <c r="B21">
         <f>B1/16</f>
-        <v>50</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -564,11 +564,11 @@
       </c>
       <c r="B22">
         <f>B1/2-B21-B20</f>
-        <v>340</v>
+        <v>435.2</v>
       </c>
       <c r="C22">
         <f>B2/2+B21*2</f>
-        <v>500</v>
+        <v>640</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -577,11 +577,11 @@
       </c>
       <c r="B23">
         <f>B1/2+B20</f>
-        <v>410</v>
+        <v>524.79999999999995</v>
       </c>
       <c r="C23">
         <f>B2/2+B21*2</f>
-        <v>500</v>
+        <v>640</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -590,11 +590,11 @@
       </c>
       <c r="B24">
         <f>B1/2-B21-B20</f>
-        <v>340</v>
+        <v>435.2</v>
       </c>
       <c r="C24">
         <f>B2/2+B21-B20*2</f>
-        <v>430</v>
+        <v>550.4</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
@@ -603,11 +603,11 @@
       </c>
       <c r="B25">
         <f>B1/2+B20</f>
-        <v>410</v>
+        <v>524.79999999999995</v>
       </c>
       <c r="C25">
         <f>B2/2+B21-B20*2</f>
-        <v>430</v>
+        <v>550.4</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -616,7 +616,7 @@
       </c>
       <c r="B28">
         <f>B1/40</f>
-        <v>20</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -625,11 +625,11 @@
       </c>
       <c r="B29">
         <f>B1/3.2</f>
-        <v>250</v>
+        <v>320</v>
       </c>
       <c r="C29">
         <f>B2/4</f>
-        <v>200</v>
+        <v>256</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -638,11 +638,11 @@
       </c>
       <c r="B30">
         <f>B1/3.2+B28</f>
-        <v>270</v>
+        <v>345.6</v>
       </c>
       <c r="C30">
         <f>B2/4</f>
-        <v>200</v>
+        <v>256</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -651,11 +651,11 @@
       </c>
       <c r="B31">
         <f>B1/3.2+B28</f>
-        <v>270</v>
+        <v>345.6</v>
       </c>
       <c r="C31">
         <f>B2/2.5</f>
-        <v>320</v>
+        <v>409.6</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -664,11 +664,11 @@
       </c>
       <c r="B32">
         <f>B1/3.2</f>
-        <v>250</v>
+        <v>320</v>
       </c>
       <c r="C32">
         <f>B2/2.5+B28</f>
-        <v>340</v>
+        <v>435.20000000000005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>